<commit_message>
Samples update for the release
</commit_message>
<xml_diff>
--- a/converted_files/835/835-all-fields.xlsx
+++ b/converted_files/835/835-all-fields.xlsx
@@ -319,7 +319,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a3a</t>
+          <t>6aaac752fd84853fa5df841c</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -541,7 +541,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:BC1"/>
+  <dimension ref="A1:AZ1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -782,40 +782,25 @@
       </c>
       <c r="AV1" s="3" t="inlineStr">
         <is>
-          <t>RemittanceDeliveryMethodReportTransmissionCode</t>
+          <t>ProviderIdentifier</t>
         </is>
       </c>
       <c r="AW1" s="3" t="inlineStr">
         <is>
-          <t>RemittanceDeliveryMethodName</t>
+          <t>FiscalPeriodDate</t>
         </is>
       </c>
       <c r="AX1" s="3" t="inlineStr">
         <is>
-          <t>RemittanceDeliveryMethodCommunicationNumber</t>
+          <t>ProviderAdjustmentReason</t>
         </is>
       </c>
       <c r="AY1" s="3" t="inlineStr">
         <is>
-          <t>ProviderIdentifier</t>
+          <t>ProviderAdjustmentReferenceIdentification</t>
         </is>
       </c>
       <c r="AZ1" s="3" t="inlineStr">
-        <is>
-          <t>FiscalPeriodDate</t>
-        </is>
-      </c>
-      <c r="BA1" s="3" t="inlineStr">
-        <is>
-          <t>ProviderAdjustmentReason</t>
-        </is>
-      </c>
-      <c r="BB1" s="3" t="inlineStr">
-        <is>
-          <t>ProviderAdjustmentReferenceIdentification</t>
-        </is>
-      </c>
-      <c r="BC1" s="3" t="inlineStr">
         <is>
           <t>ProviderAdjustmentAmount</t>
         </is>
@@ -1876,7 +1861,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a9b</t>
+          <t>6aaac752fd84853fa5df847f</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2574,7 +2559,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a9b</t>
+          <t>6aaac752fd84853fa5df847f</t>
         </is>
       </c>
       <c r="B3"/>
@@ -2838,7 +2823,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a9b</t>
+          <t>6aaac752fd84853fa5df847f</t>
         </is>
       </c>
       <c r="B4"/>
@@ -3102,7 +3087,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a9b</t>
+          <t>6aaac752fd84853fa5df847f</t>
         </is>
       </c>
       <c r="B5"/>
@@ -3366,7 +3351,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a9b</t>
+          <t>6aaac752fd84853fa5df847f</t>
         </is>
       </c>
       <c r="B6"/>
@@ -3614,7 +3599,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a9b</t>
+          <t>6aaac752fd84853fa5df847f</t>
         </is>
       </c>
       <c r="B7"/>
@@ -3908,7 +3893,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>6a68fd2aaa71f5c1ede91a9b</t>
+          <t>6aaac752fd84853fa5df847f</t>
         </is>
       </c>
       <c r="B8"/>

</xml_diff>

<commit_message>
Updated 835 Excel examples
</commit_message>
<xml_diff>
--- a/converted_files/835/835-all-fields.xlsx
+++ b/converted_files/835/835-all-fields.xlsx
@@ -6,9 +6,9 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Transactions" r:id="rId3" sheetId="1"/>
-    <sheet name="ProviderAdjustments" r:id="rId4" sheetId="2"/>
-    <sheet name="Service Lines" r:id="rId5" sheetId="3"/>
+    <sheet name="Remittances" r:id="rId3" sheetId="1"/>
+    <sheet name="Provider Adjustments" r:id="rId4" sheetId="2"/>
+    <sheet name="Claims and Service Lines" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
@@ -319,7 +319,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df841c</t>
+          <t>6ad90888b0eac4437b305abc</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1861,7 +1861,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df847f</t>
+          <t>6ad90888b0eac4437b305b1f</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df847f</t>
+          <t>6ad90888b0eac4437b305b1f</t>
         </is>
       </c>
       <c r="B3"/>
@@ -2823,7 +2823,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df847f</t>
+          <t>6ad90888b0eac4437b305b1f</t>
         </is>
       </c>
       <c r="B4"/>
@@ -3087,7 +3087,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df847f</t>
+          <t>6ad90888b0eac4437b305b1f</t>
         </is>
       </c>
       <c r="B5"/>
@@ -3351,7 +3351,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df847f</t>
+          <t>6ad90888b0eac4437b305b1f</t>
         </is>
       </c>
       <c r="B6"/>
@@ -3599,7 +3599,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df847f</t>
+          <t>6ad90888b0eac4437b305b1f</t>
         </is>
       </c>
       <c r="B7"/>
@@ -3893,7 +3893,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>6aaac752fd84853fa5df847f</t>
+          <t>6ad90888b0eac4437b305b1f</t>
         </is>
       </c>
       <c r="B8"/>

</xml_diff>